<commit_message>
fix: align release artifacts and remove exposed credential
</commit_message>
<xml_diff>
--- a/outputs/tables/repeat_purchase_90d_analysis.xlsx
+++ b/outputs/tables/repeat_purchase_90d_analysis.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3b05011208104af6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="Rbd625bbd6fbf4bd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Driver Model" sheetId="3" r:id="R3beb79c681e84948"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Rates" sheetId="4" r:id="R2d8a16388b154085"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="5" r:id="R1ea5bead24384680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcab4edeeb60b45e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R598f14fdb51b4c3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Driver Model" sheetId="3" r:id="R34bc49b3ec734330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Rates" sheetId="4" r:id="Ra90b67f1d77844e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="5" r:id="R229dcab20f6c4d8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13571dbd559c4641"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd6052509ae2f4c62"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1288,7 +1288,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69c3e75ca7ae4a21"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6e50dcdf9c84b21"/>
 </x:worksheet>
 </file>
 
@@ -1493,7 +1493,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9916009a9b5a4d49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72f482d997454543"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1973,7 +1973,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bfa50634aca4350"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7426186c8f544370"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2933,7 +2933,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R792269a406974452"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd8401ce9fc94f8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3004,12 +3004,12 @@
         <x:v>Controls right-censoring at the end of the dataset</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="7" ht="48" hidden="0" customHeight="1">
       <x:c r="A7" s="65" t="str">
         <x:v>Repeat purchase</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Second delivered order occurs within 90 days of first delivered order, inclusive</x:v>
+        <x:v>Second delivered order occurs on calendar days 1–90 after the first delivered order; same-day orders are excluded, and the earliest qualifying cross-day order is used.</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>src/analyze_repeat_purchase.py</x:v>

</xml_diff>